<commit_message>
ajout doc pdf + maquette png
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_MaresJulien_P_Appro1.xlsx
+++ b/Journal-de-Travail_MaresJulien_P_Appro1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px50vpm\Documents\GitHub\P_Bibliothèque\P_Appro1_Bibliotheque\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F714C7C-BE3B-4EE2-B625-C4FDC62C8AAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06221EDA-74CD-412D-8198-5F7AB2EED94F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -5798,7 +5798,9 @@
         <f>IF(ISBLANK(B60),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B60))</f>
         <v>11</v>
       </c>
-      <c r="B65" s="84"/>
+      <c r="B65" s="84">
+        <v>46094</v>
+      </c>
       <c r="C65" s="85">
         <v>2</v>
       </c>
@@ -5818,7 +5820,9 @@
         <f>IF(ISBLANK(B61),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B61))</f>
         <v>11</v>
       </c>
-      <c r="B66" s="84"/>
+      <c r="B66" s="84">
+        <v>46094</v>
+      </c>
       <c r="C66" s="85"/>
       <c r="D66" s="86">
         <v>10</v>

</xml_diff>